<commit_message>
Integrate revised Spanish titles into complete publisher and material previews
</commit_message>
<xml_diff>
--- a/materials/西语/assets_es_20261106_two_daily/西语标题与封面对应表.xlsx
+++ b/materials/西语/assets_es_20261106_two_daily/西语标题与封面对应表.xlsx
@@ -514,16 +514,16 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>¡Su banco inventó deudas de sus abuelos muertos! Este abogado destapó la estafa del pueblo</t>
+          <t>¡El banco cobró deudas de sus abuelos muertos! Él destapó una estafa que atrapó a todo el pueblo</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>银行伪造已故祖辈欠款，律师揭穿全村骗局</t>
+          <t>银行竟追讨已故祖辈的欠款！他一路查下去，揭开了坑害全村的骗局！</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -557,16 +557,16 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>¡Invadieron su mundo! Él invocó a 3000 maestros y llevó la batalla al reino de los espectros</t>
+          <t>¡Los espectros invadieron su país! Activó su sistema e invocó a 3000 maestros para contraatacar</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>诡异入侵，他召唤三千祖师反攻</t>
+          <t>诡异竟入侵他的国家！他激活系统，召唤三千祖师直接反攻！</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -600,16 +600,16 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>¡El muerto señaló a su asesino! Un artesano milenario reveló la traición con sus agujas</t>
+          <t>¡El muerto levantó la mano y señaló al asesino! Un artesano de mil años lo logró con sus agujas</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>千年缝尸匠用针破邪术，逝者指出凶手</t>
+          <t>死人竟抬手指出凶手！这个活了千年的缝尸匠，用几根针做到了！</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -643,16 +643,16 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>¡De eunuco a regente! Su sistema del harén lo convirtió en el hombre más poderoso del reino</t>
+          <t>¡Despertó como eunuco con un sistema! El emperador quiso matarlo y él terminó como regente</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>后宫签到系统，让底层太监逆袭摄政王</t>
+          <t>一觉醒来成了太监，竟还自带系统！皇帝想杀他，他却一路当上摄政王！</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -686,16 +686,16 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>¡El masajista ocultaba un pasado temible! Volvió para romper la red de apuestas de la ciudad</t>
+          <t>¡Un masajista contra toda una red de apuestas! Su familia podía estar en manos de los culpables</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>足疗店主重出江湖，追查地下赌局</t>
+          <t>一个足疗工，要对抗整张地下赌网！他的家人可能也落在了幕后黑手手里！</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -729,16 +729,16 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>¡Lo convirtieron en gallo! Con un sistema de fama evolucionó en fénix y salvó su zoológico</t>
+          <t>¡Lo traicionaron y acabó convertido en gallo! Su sistema de fama lo hizo evolucionar en fénix</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>被害变成芦花鸡，靠声望系统进化凤凰</t>
+          <t>遭人背叛后，他竟变成一只鸡！靠声望系统一路进化，最终化身凤凰！</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -772,16 +772,16 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>¡Humillaron al abuelo equivocado! Su sello cayó y el inmortal de la espada despertó</t>
+          <t>¡Humillaron a un anciano y golpearon a su nieto! Era un inmortal sellado durante 50 años</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>嘲讽老人，却触发剑仙封印解除</t>
+          <t>他们羞辱老人，还打伤他的孙子！却不知眼前之人，是自封修为五十年的仙人！</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -815,16 +815,16 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>¡Llevaba 500 años ciego! Sus alumnos desafiaron a los dioses y él abrió los ojos como un santo</t>
+          <t>¡Enseñó 500 años sin poder ver! Sus alumnos enfrentaron a los dioses y él por fin abrió los ojos</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>失明五百年，弟子逆伐诸天后师尊睁眼成圣</t>
+          <t>他双目失明，却传道整整五百年！弟子们逆战诸神，他终于睁开双眼！</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -858,16 +858,16 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>¡El incienso ocultaba una trampa! Entró en la casa sellada para descubrir qué pasó con su novia</t>
+          <t>¡Oyó risas de mujer en una casa vacía! Buscaba a su novia y el incienso lo llevó a una trampa</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>封锁老屋的香料藏着骗局，他追查失踪女友</t>
+          <t>空屋里竟传来女人的声音！他追查失踪女友，却发现香火背后藏着陷阱！</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -901,16 +901,16 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>¡Renació como pulpo y predijo el Mundial! Su sistema destapó una amenaza en el fondo del mar</t>
+          <t>¡Despertó como pulpo con un sistema de predicción! Acertó los partidos y volvió rico a un endeudado</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>重生成章鱼，预言世界杯并揭穿海底黑幕</t>
+          <t>一觉醒来变成章鱼，竟绑定预言系统！精准预测球赛，让负债青年一夜暴富！</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -944,16 +944,16 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>¡Sus amadas lo traicionaron! Renació como renacuajo y volvió convertido en Emperador Rana</t>
+          <t>¡Lo mataron y renació como renacuajo! Devoró, evolucionó y volvió como Emperador Rana para vengarse</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>道侣背叛后重生成蝌蚪，进化蛙帝归来清算</t>
+          <t>他被害后竟重生成蝌蚪！靠吞噬不断进化，再归来时已是复仇的蛙帝！</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -987,16 +987,16 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>¡Su vecino inundó su casa! Construyó un muro legal y la siguiente lluvia cambió todo</t>
+          <t>¡Su vecino desvió el agua y arruinó su casa! Él construyó un muro y la lluvia hizo el resto</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>恶邻改排水害人，他依法建墙让局势逆转</t>
+          <t>恶邻改动排水，害他家被淹！他建起一道墙，下一场大雨让局势彻底逆转！</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1030,16 +1030,16 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>¡Les pagó los estudios y lo abandonaron al enfermar! Sus abusos tendrán consecuencias</t>
+          <t>¡Les pagó los estudios y aun enfermo quisieron aprovecharse de él! Esta vez respondió con la ley</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>资助他人却病中遭背弃，他用法律反击贪婪</t>
+          <t>他资助他们读书，自己病重时却仍遭算计！这一次，他选择用法律讨回公道！</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1073,16 +1073,16 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>¡Cambió las espadas por exámenes! Su sistema convirtió una secta débil en la más poderosa</t>
+          <t>¡En vez de practicar con espadas, los puso a hacer exámenes! Su secta acabó venciendo a las demás</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>系统加科学刷题，弱小宗门逆袭登顶</t>
+          <t>别人练剑，他却让弟子做试卷！这个宗门最后竟打败了其他所有宗门！</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1116,16 +1116,16 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>¡El muñeco de su esposa escondía una traición! Él tendió la trampa que salvó su empresa</t>
+          <t>¡Su esposa se encerraba con un muñeco! Instaló una cámara y descubrió la traición de su mejor amigo</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>妻子的人偶藏着背叛，他布局保住公司</t>
+          <t>妻子竟总和人偶独处一室！他装上监控暗查，却发现最好的兄弟也卷入了背叛！</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1159,16 +1159,16 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>¡Perdieron ocho duelos! Él eligió a un mortal que ocultaba una fuerza capaz de salvar su nación</t>
+          <t>¡Tras ocho derrotas, convocó a un general mortal! Su forma real era la última esperanza del país</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>连败八场后，他召唤隐藏强者守护国运</t>
+          <t>连败八场后，他竟召唤一个凡人将领！而将领的真正形态，成了国家最后的希望！</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1202,16 +1202,16 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>¡Lo despreciaron sin saber que era rico! Rescató a su novia y dejó de ceder ante su familia</t>
+          <t>¡Exigieron 300 mil yuanes por su novia! Él la rescató: habían humillado a un millonario</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>隐藏身家的富豪救出新娘，不再向贪婪家人让步</t>
+          <t>他们开口就要三十万彩礼！他救走新娘，对方却不知自己羞辱的竟是个富豪！</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1245,16 +1245,16 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>¡Un artesano con sistema de ferretería! Sus herramientas dejaron en ridículo a los espadachines</t>
+          <t>¡Activó un sistema de ferretería entre inmortales! Usó un cañón de agua contra sus espadas</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>落魄匠师绑定五金系统，用现代工具对战剑修</t>
+          <t>穿越修仙世界，他竟激活五金店系统！别人御剑，他直接搬出高压水炮！</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1288,16 +1288,16 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>¡Entró al monte por su madre! Los cazadores de tumbas lo habían convertido en su cebo</t>
+          <t>¡Entró a cazar bajo la luna roja por su madre! Lo estaban usando de cebo para encontrar una tumba</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>为母亲进山求药费，却成盗墓贼寻墓诱饵</t>
+          <t>为救母亲，他冒险在血月之夜进山打猎！却被人当成寻找古墓的活饵！</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1331,16 +1331,16 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>¡Cuatro compañeras lo traicionaron! Él dominó a las bestias y ellas perdieron su poder</t>
+          <t>¡Cuatro hermanas de secta lo traicionaron! Él ascendió con sus bestias y ellas quedaron mortales</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>四位师姐背叛，他转修御兽崛起令她们后悔</t>
+          <t>四位师姐联手背叛了他！他靠御兽之道飞升，她们却沦为凡人！</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>

</xml_diff>